<commit_message>
act y se cambia de raiz
</commit_message>
<xml_diff>
--- a/new-stats/aarhus.xlsx
+++ b/new-stats/aarhus.xlsx
@@ -1903,22 +1903,62 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>06/04/2026</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Viborg</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Aarhus</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="M26" t="n">
+        <v>13</v>
+      </c>
+      <c r="N26" t="n">
+        <v>11</v>
+      </c>
+      <c r="O26" t="n">
+        <v>5</v>
+      </c>
+      <c r="P26" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>

</xml_diff>

<commit_message>
act y cambio en proyeccion remates
</commit_message>
<xml_diff>
--- a/new-stats/aarhus.xlsx
+++ b/new-stats/aarhus.xlsx
@@ -2019,22 +2019,62 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Midtjylland</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Aarhus</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="M28" t="n">
+        <v>15</v>
+      </c>
+      <c r="N28" t="n">
+        <v>12</v>
+      </c>
+      <c r="O28" t="n">
+        <v>6</v>
+      </c>
+      <c r="P28" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>

</xml_diff>